<commit_message>
Fix 34 URL/Instagram/email errors after manual verification
Corrections applied per web research:
- nylon.coffee (was nyloncoffee.sg)
- tionghoe.com, @tionghoespecialtycoffee
- homegroundcoffeeroasters.com, @homeground.coffee
- @strangersreu (was @strangersreunion)
- Nana Coffee Roasters + nanacoffeeroasters.com
- ceresiacoffeeroasters.com
- kaizencoffee.com
- monsoontea.co.th
- arabianteahouse.com
- thesumofusdubai.com
- stompinggrounds.ae, @stompinggroundsdxb
- Various email corrections

https://claude.ai/code/session_018H7qJLrHHVqqsfGNGj5Jik
</commit_message>
<xml_diff>
--- a/hojicha_export_targets.xlsx
+++ b/hojicha_export_targets.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>https://nyloncoffee.sg</t>
+          <t>https://nylon.coffee</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -596,7 +596,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>info@nyloncoffee.sg</t>
+          <t>hello@nyloncoffee.com</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>info@commonmancoffeeroasters.com</t>
+          <t>info@cmcroasters.com</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -838,17 +838,17 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>https://www.tionghoecoffee.com</t>
+          <t>https://tionghoe.com</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>@tionghoecoffee</t>
+          <t>@tionghoespecialtycoffee</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>tionghoe@gmail.com</t>
+          <t>hello@tionghoe.com</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -880,17 +880,17 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>https://homegroundcoffee.sg</t>
+          <t>https://homegroundcoffeeroasters.com</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>@homegroundcoffeeroasters</t>
+          <t>@homeground.coffee</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>hello@homegroundcoffee.sg</t>
+          <t>hello@homegroundcoffeeroasters.com</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -927,12 +927,12 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>@strangersreunion</t>
+          <t>@strangersreu</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>hello@strangersreunion.com</t>
+          <t>enquiries@strangersreunion.com</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>reservations@odetterestaurant.com</t>
+          <t>enquiry@odetterestaurant.com</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
@@ -2444,7 +2444,7 @@
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>hello@teakha.com</t>
+          <t>discover@teakha.com</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
@@ -3148,7 +3148,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t>https://www.ceresiacoffee.com</t>
+          <t>https://ceresiacoffeeroasters.com</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>info@ceresiacoffee.com</t>
+          <t>info@ceresiacoffeeroasters.com</t>
         </is>
       </c>
       <c r="H63" s="5" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Nana Roasters</t>
+          <t>Nana Coffee Roasters</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -3232,17 +3232,17 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>https://www.nanaroasters.com</t>
+          <t>https://nanacoffeeroasters.com</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>@nanaroasters</t>
+          <t>@nanacoffeeroasters</t>
         </is>
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>hello@nanaroasters.com</t>
+          <t>info@nanacoffeeroasters.com</t>
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr">
@@ -3274,7 +3274,7 @@
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>https://www.inkandlioncafe.com</t>
+          <t>https://www.facebook.com/inkandlioncafe</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
@@ -3284,7 +3284,7 @@
       </c>
       <c r="G66" s="9" t="inlineStr">
         <is>
-          <t>hello@inkandlioncafe.com</t>
+          <t>inkandlioncafe@gmail.com</t>
         </is>
       </c>
       <c r="H66" s="9" t="inlineStr">
@@ -3400,7 +3400,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t>https://www.kaizencoffeeco.com</t>
+          <t>https://www.kaizencoffee.com</t>
         </is>
       </c>
       <c r="F69" s="5" t="inlineStr">
@@ -3410,7 +3410,7 @@
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>hello@kaizencoffeeco.com</t>
+          <t>info@kaizencoffee.com</t>
         </is>
       </c>
       <c r="H69" s="5" t="inlineStr">
@@ -3484,7 +3484,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t>https://www.waldenwoodsbkk.com</t>
+          <t>https://www.instagram.com/waldenwoodsbangkok</t>
         </is>
       </c>
       <c r="F71" s="5" t="inlineStr">
@@ -3494,7 +3494,7 @@
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>hello@waldenwoodsbkk.com</t>
+          <t>waldenwoodsbangkok@gmail.com</t>
         </is>
       </c>
       <c r="H71" s="5" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>https://www.monsoontea.co</t>
+          <t>https://www.monsoontea.co.th</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>info@monsoontea.co</t>
+          <t>info@monsoontea.co.th</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4534,7 +4534,7 @@
       </c>
       <c r="E96" s="11" t="inlineStr">
         <is>
-          <t>https://www.arabianteahouse.ae</t>
+          <t>https://arabianteahouse.com</t>
         </is>
       </c>
       <c r="F96" s="11" t="inlineStr">
@@ -4544,7 +4544,7 @@
       </c>
       <c r="G96" s="11" t="inlineStr">
         <is>
-          <t>info@arabianteahouse.ae</t>
+          <t>info@arabianteahouse.com</t>
         </is>
       </c>
       <c r="H96" s="11" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="E98" s="11" t="inlineStr">
         <is>
-          <t>https://www.thesumofus.com</t>
+          <t>https://www.thesumofusdubai.com</t>
         </is>
       </c>
       <c r="F98" s="11" t="inlineStr">
@@ -4628,7 +4628,7 @@
       </c>
       <c r="G98" s="11" t="inlineStr">
         <is>
-          <t>hello@thesumofus.com</t>
+          <t>hello@thesumofusdubai.com</t>
         </is>
       </c>
       <c r="H98" s="11" t="inlineStr">
@@ -4660,17 +4660,17 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t>https://www.stompinggrounds.coffee</t>
+          <t>https://www.stompinggrounds.ae</t>
         </is>
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>@stompinggrounds.ae</t>
+          <t>@stompinggroundsdxb</t>
         </is>
       </c>
       <c r="G99" s="5" t="inlineStr">
         <is>
-          <t>info@stompinggrounds.coffee</t>
+          <t>info@stompinggrounds.ae</t>
         </is>
       </c>
       <c r="H99" s="5" t="inlineStr">

</xml_diff>